<commit_message>
Finalize CRM portfolio demo and activity log validation
</commit_message>
<xml_diff>
--- a/output/Customer_Data_Management_Workbook.xlsx
+++ b/output/Customer_Data_Management_Workbook.xlsx
@@ -21,7 +21,6 @@
     <definedName name="Industries">'04_Validation_Lists'!$C$2:$C$10</definedName>
     <definedName name="LeadSources">'04_Validation_Lists'!$D$2:$D$7</definedName>
     <definedName name="Priorities">'04_Validation_Lists'!$E$2:$E$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'06_Activity_Log'!$A$4:$F$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -193,8 +192,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerDatabaseTable" displayName="CustomerDatabaseTable" ref="A4:J4" headerRowCount="1">
-  <autoFilter ref="A4:J4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerDatabaseTable" displayName="CustomerDatabaseTable" ref="A4:J5" headerRowCount="1">
+  <autoFilter ref="A4:J5"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Customer ID"/>
     <tableColumn id="2" name="First Name"/>
@@ -212,8 +211,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A4:F4" headerRowCount="1">
-  <autoFilter ref="A4:F4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A4:F5" headerRowCount="1">
+  <autoFilter ref="A4:F5"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Activity ID"/>
     <tableColumn id="2" name="Timestamp"/>
@@ -1185,7 +1184,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>